<commit_message>
Project test123 is saved.
</commit_message>
<xml_diff>
--- a/test123/Main.xlsx
+++ b/test123/Main.xlsx
@@ -193,7 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="50">
   <si>
     <t>Rule</t>
   </si>
@@ -1045,7 +1045,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:G29"/>
+  <dimension ref="B3:G35"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="1" width="2.85546875"/>
@@ -1178,26 +1178,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" t="s" s="1">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" t="s" s="1">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" t="s" s="1">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" t="s" s="1">
-        <v>26</v>
-      </c>
-    </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
     <row r="18">
       <c r="B18" s="1" t="s">
         <v>44</v>
@@ -1269,6 +1253,31 @@
       </c>
       <c r="C29" t="s" s="0">
         <v>32</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="s" s="1">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="s" s="1">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="s" s="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="s" s="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="1" t="n">
+        <v>234234.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>